<commit_message>
fixed the round error
</commit_message>
<xml_diff>
--- a/test/Grades.xlsx
+++ b/test/Grades.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
   <si>
     <t>Name</t>
   </si>
@@ -47,6 +47,12 @@
   </si>
   <si>
     <t>Jasper</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
   </si>
   <si>
     <t>C</t>
@@ -421,7 +427,7 @@
         <v>91</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>85</v>
       </c>
       <c r="G2" t="s">
         <v>11</v>
@@ -444,10 +450,10 @@
         <v>68</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>75</v>
       </c>
       <c r="G3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -467,7 +473,7 @@
         <v>74</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>86.3</v>
       </c>
       <c r="G4" t="s">
         <v>11</v>
@@ -490,10 +496,10 @@
         <v>80</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>65.3</v>
       </c>
       <c r="G5" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -513,10 +519,10 @@
         <v>70</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>76.7</v>
       </c>
       <c r="G6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>